<commit_message>
Incluir filas con FIN (KM) en blanco tal cual Excel
- Si FIN está vacío: incluir cuando INICIO cae dentro del tramo
- Si FIN tiene valor: mantener filtro estricto (actividad contenida)
- FIN en blanco se exporta vacío en CSV/Excel/JSON
- Total: 866 registros (+124 respecto a versión anterior)

Co-authored-by: NicolasCutire <NicolasCutire@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/extracted/reports/tramos_filtrado_estricto/tramo_146+500_146+520.xlsx
+++ b/extracted/reports/tramos_filtrado_estricto/tramo_146+500_146+520.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -485,7 +485,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Filtro estricto: INICIO (KM) y FIN (KM) contenidos en el tramo | Total registros: 21</t>
+          <t>Filtro: FIN completo contenido en tramo; FIN en blanco si INICIO cae en tramo | Total registros: 26</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Año 2020 (2 registros)</t>
+          <t>Año 2020 (5 registros)</t>
         </is>
       </c>
       <c r="B18" s="2" t="n"/>
@@ -924,209 +924,213 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Limpieza de carril/pista y bermas T2</t>
+          <t>Reposición de Cuneta</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>2020-03-19</t>
+          <t>2020-01-06</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>146+500</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>146+520</t>
-        </is>
-      </c>
+          <t>146+510</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n">
-        <v>72</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
+          <t>Reposición de Cuneta</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>2020-01-06</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>146+520</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Limpieza de carril/pista y bermas T2</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>2020-03-19</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>146+500</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>146+520</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
           <t>Limpieza Manual de Cabezal de Alcantarilla T2</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>2020-12-01</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>2020-04-23</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>146+520</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>146+520</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Año 2021 (2 registros)</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>INICIO (KM)</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>FIN (KM)</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>METRADO</t>
-        </is>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t>Limpieza Manual de Cabezal de Alcantarilla T2</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>2020-12-01</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>146+520</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>146+520</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Año 2021 (2 registros)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>INICIO (KM)</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>FIN (KM)</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>METRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
           <t>Limpieza Manual de Cuneta de Vía T2</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>2021-04-03</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>146+500</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>146+510</t>
         </is>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F27" s="5" t="n">
         <v>10</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Limpieza Manual de Cabezal de Alcantarilla T2</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>2021-12-06</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>146+520</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>146+520</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Año 2022 (1 registros)</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>INICIO (KM)</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>FIN (KM)</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>METRADO</t>
-        </is>
       </c>
     </row>
     <row r="28">
@@ -1142,7 +1146,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>2022-11-28</t>
+          <t>2021-12-06</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -1156,13 +1160,13 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Año 2024 (2 registros)</t>
+          <t>Año 2022 (1 registros)</t>
         </is>
       </c>
       <c r="B29" s="2" t="n"/>
@@ -1216,95 +1220,95 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
+          <t>2022-11-28</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>146+520</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>146+520</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Año 2024 (2 registros)</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>INICIO (KM)</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>FIN (KM)</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>METRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Limpieza Manual de Cabezal de Alcantarilla T2</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
           <t>2024-04-13</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>146+510</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>146+514</t>
         </is>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="F34" s="5" t="n">
         <v>12</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Limpieza Manual de Cabezal de Alcantarilla T2</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>2024-06-28</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>146+520</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>146+520</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Año 2025 (4 registros)</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>INICIO (KM)</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>FIN (KM)</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>METRADO</t>
-        </is>
       </c>
     </row>
     <row r="35">
@@ -1320,124 +1324,295 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>2025-05-23</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>146+510</t>
+          <t>146+520</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>146+510</t>
+          <t>146+520</t>
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Limpieza Manual de Cabezal de Alcantarilla T2</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>2025-06-09</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>146+510</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>146+514</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="n">
-        <v>14</v>
-      </c>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Año 2025 (5 registros)</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>Limpieza Manual de Cabezal de Alcantarilla T2</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>2025-06-10</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>146+510</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>146+514</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="n">
-        <v>14</v>
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>INICIO (KM)</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>FIN (KM)</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>METRADO</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
+          <t>Limpieza Manual de Cabezal de Alcantarilla T2</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>2025-03-24</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>146+500</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="5" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Limpieza Manual de Cabezal de Alcantarilla T2</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>2025-05-23</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>146+510</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>146+510</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Limpieza Manual de Cabezal de Alcantarilla T2</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>2025-06-09</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>146+510</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>146+514</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Limpieza Manual de Cabezal de Alcantarilla T2</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>2025-06-10</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>146+510</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>146+514</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
           <t>Limpieza Manual de Cuerpo de Alcantarilla T2</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>2025-08-28</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>146+500</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>146+505</t>
         </is>
       </c>
-      <c r="F38" s="5" t="n">
+      <c r="F42" s="5" t="n">
         <v>14</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Año 2026 (1 registros)</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>INICIO (KM)</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>FIN (KM)</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>METRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Limpieza mecanizada de cabezal de alcantarilla T2</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>146+520</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A36:F36"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A32:F32"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>